<commit_message>
Add heat-order drag sorting in RatioFix STEP 2; fix Step1 tolerance
- Heat chips draggable (HTML5 DnD): DOM order commits to characters,
  resets confirm state and auto-balance snapshot; arrow micro-adjust kept
- Step 1 fatal parse errors render to error panel instead of silent fail;
  total points input strictly validated as positive integer
- Cross-table total-price tolerance fixed to 0.005 yuan (user-entered
  average rounding vs internal full precision)
- Smoke test 28/28: prices stay bound to role names across drag, balance,
  Step 3 sheet, downloaded xlsx and Step 5 final table (not old order)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/演示/原排表吧唧.xlsx
+++ b/演示/原排表吧唧.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RenSheet\演示\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD3C167-6D8C-40BB-A63D-E1234ABB2141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8457DD4B-F3C8-4A68-8089-9FBDD46B17A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3040" yWindow="60" windowWidth="14420" windowHeight="15220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="13">
   <si>
     <t>吧唧</t>
   </si>
@@ -72,6 +72,10 @@
   </si>
   <si>
     <t>梶莲</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>C</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -543,7 +547,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -569,7 +573,7 @@
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
         <v>9</v>
@@ -595,7 +599,7 @@
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D9" t="s">
         <v>9</v>
@@ -621,7 +625,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
         <v>9</v>
@@ -647,7 +651,7 @@
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
         <v>9</v>

</xml_diff>